<commit_message>
Add notifications, access controls, import undo, and fresh-start tooling
- Add notification and account notice models, controller, routes, and
  services, plus an update email template and header notification UI
- Add program head and consultant access services with an AccessChip
  component and consultant courses table
- Add import undo (routes, utils, UndoUploadButton, undo toast) and
  fresh-start utilities with tests
- Update controllers, routes, invitations, mailer, and role utilities
- Refresh sample upload files and README
</commit_message>
<xml_diff>
--- a/sample-uploads/sample_course_assignments.xlsx
+++ b/sample-uploads/sample_course_assignments.xlsx
@@ -1,52 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Course Assignments" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Course Assignments" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -65,13 +42,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -396,172 +440,448 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col width="12.83203125" customWidth="1" min="1" max="1"/>
+    <col width="44.83203125" customWidth="1" min="2" max="2"/>
+    <col width="13.83203125" customWidth="1" min="3" max="3"/>
+    <col width="22.83203125" customWidth="1" min="4" max="4"/>
+    <col width="30.83203125" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>COURSE NO.</v>
-      </c>
-      <c r="B1" t="str">
-        <v>COURSE OFFERING</v>
-      </c>
-      <c r="C1" t="str">
-        <v>YEAR LEVEL</v>
-      </c>
-      <c r="D1" t="str">
-        <v>CONTRIBUTORS</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>COURSE NO.</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>COURSE OFFERING</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>YEAR LEVEL</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>LEAD FACULTY</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>CONTRIBUTORS</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>BIT101</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Introduction to Computing</v>
-      </c>
-      <c r="C2" t="str">
-        <v>1st Year</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Bianca G. Reyes; Bowen Higgins</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BIT111L</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Introduction to Computing</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FIRST YEAR</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Monica Norton</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Bianca G. Reyes</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>BIT102</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Computer Programming 1</v>
-      </c>
-      <c r="C3" t="str">
-        <v>1st Year</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Bowen Higgins</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BIT112L</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fundamentals of Programming</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FIRST YEAR</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bowen Higgins</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Olivia Vance</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>BIT201</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Database Systems</v>
-      </c>
-      <c r="C4" t="str">
-        <v>2nd Year</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Marceline Avila; Dennis Ignacio</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GEE-LITE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Living in the IT Era</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FIRST YEAR</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Christine A. Dizon</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>BIT202</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Object-Oriented Programming</v>
-      </c>
-      <c r="C5" t="str">
-        <v>2nd Year</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Christine A. Dizon</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BIT211L</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Database Management (Info Mgt) 1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SECOND YEAR</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Marceline Avila</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>BIT205</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Data Structures and Algorithms</v>
-      </c>
-      <c r="C6" t="str">
-        <v>2nd Year</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Dennis Ignacio</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BIT212L</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Web Development 1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SECOND YEAR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Saige Fuentes</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <v>BIT301</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Web Development</v>
-      </c>
-      <c r="C7" t="str">
-        <v>3rd Year</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Saige Fuentes; Harold T. Lim</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BIT213L</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Object-Oriented Programming</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SECOND YEAR</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Dennis Ignacio</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Harold T. Lim</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
-        <v>BIT303</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Software Engineering</v>
-      </c>
-      <c r="C8" t="str">
-        <v>3rd Year</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Danny B. Casimero</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BIT214L</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Networking and Communications 1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SECOND YEAR</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Michael R. Lee</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
-        <v>BIT304</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Network Security</v>
-      </c>
-      <c r="C9" t="str">
-        <v>3rd Year</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Michael R. Lee</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BIT215L</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Social Issues and Professional Practice</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SECOND YEAR</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Kristine San Lorenzo</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
-        <v>BIT313L</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Human and Computer Interaction</v>
-      </c>
-      <c r="C10" t="str">
-        <v>3rd Year</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Harold T. Lim</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BIT311L</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Platform Technologies</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>THIRD YEAR</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Danny B. Casimero</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
-        <v>BIT401</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Capstone Project 1</v>
-      </c>
-      <c r="C11" t="str">
-        <v>4th Year</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Danny B. Casimero</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BIT312L</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Integrative Programming and Technologies</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>THIRD YEAR</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Harold T. Lim</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BIT313L</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Human Computer Interaction</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>THIRD YEAR</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Margaret Hamilton</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Monica Norton</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BIT314L</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Information Systems</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>THIRD YEAR</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Sarah Jenkins</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BIT315L</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Quantitative Methods</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>THIRD YEAR</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Thomas Bayes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BIT316L</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Fundamentals of IT Project Management</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>THIRD YEAR</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>John Backus</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MATH311L</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Statistics</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>THIRD YEAR</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Alan Turing</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BIT411L</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Information Assurance and Security 2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FOURTH YEAR</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>June Arreb Danila</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BIT412L</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Capstone Project 2</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>FOURTH YEAR</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Danny B. Casimero</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Kristine San Lorenzo</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>